<commit_message>
Fix Fleet Mode remote monitoring cost
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="R8bf4c06ade794b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="R2db3ef73579642d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="Ra88f01ce45944d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="Rdfbdc73c211b427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="R9547b2eb1ab541b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturing Campus Database" sheetId="7" r:id="R4dcef40e5fd54516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing Campus Database" sheetId="8" r:id="Rcaf809a7779a4659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="R52a9d9dabfdc4dda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="R22ff496b417a4c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="R81e91fe00cd54426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="R4e8267f984e44e93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="Ra005a06c05fa4ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturing Campus Database" sheetId="7" r:id="R0c6fb6fe3f9443eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing Campus Database" sheetId="8" r:id="Re233407a16cc488f"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CRF">#REF!</x:definedName>
@@ -3137,9 +3137,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SER Number of Operators Per Shift</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Operator headcount per reactor monitored</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SER Security Staff Per Shift</x:t>
@@ -22968,18 +22965,18 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R64c5caf151044e7d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="Rae546124b40b4458"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="R789b5e6cf2374936"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="Ra8b6fc3042fa465b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="Rfc32f0bb4c544c0b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U106" r:id="R304dae256a824bdb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U117" r:id="R93220db8814a4bcc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U127" r:id="R8499c1606bbb4587"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U128" r:id="R920b1d982ec241a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U132" r:id="R8d2b24e34ee84b10"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U133" r:id="R5ccef4f1f3304acb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U166" r:id="R9f0bff6f66f1406e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R7ed5c52c791844ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="R0acfdc5f00cd4ce4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="R5396824f765949d6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="Ra383cd6292514a11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="Rb72f3fa1204e454b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U106" r:id="R9f97213bb1894a5a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U117" r:id="R02e29dab23c54eeb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U127" r:id="Rd484ac8b64754e91"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U128" r:id="R5eeedc6b469f4d83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U132" r:id="R3d9388127e1a44dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U133" r:id="R46ced60c15d04f34"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U166" r:id="Rc38972d7745c49db"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -25824,7 +25821,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62a63c5f0fbd40fb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f45ce389a984881"/>
 </x:worksheet>
 </file>
 
@@ -31507,12 +31504,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R0c9bf763590f4ebb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="Rbee77094648a45ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U66" r:id="Rd87deb7bc44645f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R146889ef723144a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="R4ee23c77680d4c4d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U66" r:id="R8f7d05aedf164762"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R573feb1f528a4ebc"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4565902e5e49fc"/>
 </x:worksheet>
 </file>
 
@@ -37222,8 +37219,8 @@
       <x:c r="E75" s="96" t="s">
         <x:v>268</x:v>
       </x:c>
-      <x:c r="F75" s="96" t="s">
-        <x:v>752</x:v>
+      <x:c r="F75" s="96" t="str">
+        <x:v>Reactors Monitored Per Operator</x:v>
       </x:c>
       <x:c r="G75" s="97">
         <x:v>1</x:v>
@@ -37329,7 +37326,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M76" s="59" t="s">
-        <x:v>753</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="N76" s="106"/>
       <x:c r="O76" s="106"/>
@@ -37486,7 +37483,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C78" s="112" t="s">
-        <x:v>754</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="D78" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37507,7 +37504,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M78" s="209" t="s">
-        <x:v>755</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="N78" s="106"/>
       <x:c r="O78" s="106"/>
@@ -37728,7 +37725,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C82" s="112" t="s">
-        <x:v>756</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="D82" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37786,7 +37783,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C83" s="112" t="s">
-        <x:v>757</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="D83" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37921,7 +37918,7 @@
         <x:v>418</x:v>
       </x:c>
       <x:c r="M85" s="96" t="s">
-        <x:v>758</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="N85" s="106"/>
       <x:c r="O85" s="106"/>
@@ -38044,7 +38041,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C87" s="112" t="s">
-        <x:v>759</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="D87" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38089,7 +38086,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C88" s="112" t="s">
-        <x:v>760</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="D88" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38099,7 +38096,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F88" s="96" t="s">
-        <x:v>761</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="G88" s="97">
         <x:v>1</x:v>
@@ -38122,12 +38119,12 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S88" s="113" t="s">
-        <x:v>762</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="T88" s="114"/>
       <x:c r="U88" s="208"/>
       <x:c r="V88" s="106" t="s">
-        <x:v>763</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="W88" s="99" t="s">
         <x:v>43</x:v>
@@ -38174,7 +38171,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C89" s="112" t="s">
-        <x:v>764</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="D89" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38184,7 +38181,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F89" s="96" t="s">
-        <x:v>765</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="G89" s="97">
         <x:v>1</x:v>
@@ -38279,7 +38276,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C90" s="112" t="s">
-        <x:v>766</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="D90" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38289,7 +38286,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F90" s="96" t="s">
-        <x:v>767</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="G90" s="97">
         <x:v>1</x:v>
@@ -38312,12 +38309,12 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S90" s="113" t="s">
-        <x:v>762</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="T90" s="114"/>
       <x:c r="U90" s="208"/>
       <x:c r="V90" s="106" t="s">
-        <x:v>763</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="W90" s="99" t="s">
         <x:v>43</x:v>
@@ -38389,7 +38386,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M91" s="113" t="s">
-        <x:v>768</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="N91" s="106"/>
       <x:c r="O91" s="106" t="s">
@@ -38504,7 +38501,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C93" s="112" t="s">
-        <x:v>769</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="D93" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38549,7 +38546,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C94" s="194" t="s">
-        <x:v>770</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="D94" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38633,7 +38630,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C95" s="194" t="s">
-        <x:v>771</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="D95" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38717,7 +38714,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C96" s="194" t="s">
-        <x:v>772</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="D96" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38801,7 +38798,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C97" s="194" t="s">
-        <x:v>773</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="D97" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -39255,13 +39252,13 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="Rb8a70f79952e47b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="R4ff9552f39b84362"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="R73bd34599c51482c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="R8b6b69680366449e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U91" r:id="R9f4aeac1775340d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="Ref510b6a5f354956"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="R96a6c4ae10ed49f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="R15030bf7d56f43fb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="R4992b1fc0893483f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U91" r:id="R95f3a41021bf450c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b7994c4f0c34f02"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdba283c3ed744199"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Fleet Mode manufacturing campus costs
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="R52a9d9dabfdc4dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="R22ff496b417a4c6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="R81e91fe00cd54426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="R4e8267f984e44e93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="Ra005a06c05fa4ded"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturing Campus Database" sheetId="7" r:id="R0c6fb6fe3f9443eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing Campus Database" sheetId="8" r:id="Re233407a16cc488f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Database" sheetId="1" r:id="R498d02ce6da54925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MARVEL_Cost" sheetId="2" r:id="R04802edbed98459f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Variables" sheetId="3" r:id="R5520748934df4174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inflation Adjustment" sheetId="4" r:id="Rdf59b7b0fb4d4b37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economics Parameters" sheetId="5" r:id="R697b68b68ae64308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturing Campus Database" sheetId="7" r:id="R33e45c08cece4b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicing Campus Database" sheetId="8" r:id="R9432f155024d4d31"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="CRF">#REF!</x:definedName>
@@ -2677,9 +2677,6 @@
     <x:t xml:space="preserve">Testing Building</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">!!! TO EQUAL PART, BUT NOT ALL, OF GENERATING SITE COST.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Warehouse</x:t>
   </x:si>
   <x:si>
@@ -2791,9 +2788,6 @@
     <x:t xml:space="preserve">MFG Guard Station Count</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Assume 50% of direct cost  - need to add handling for this in MOUSE script.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Operators (Testing Only)</x:t>
   </x:si>
   <x:si>
@@ -2830,15 +2824,9 @@
     <x:t xml:space="preserve">Continuing Education and Staff Retraining</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Assume 2% of sum of accounts 711 through 715 - need to add handling for this in MOUSE script.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Management Staff</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Assume 7.5% of sum of accounts 711 through 715 - need to add handling for this in MOUSE script.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Manfuacturing Building Staff</x:t>
   </x:si>
   <x:si>
@@ -2851,21 +2839,12 @@
     <x:t xml:space="preserve">Operating Chemicals and Lubricants (Except Manufacturing and Fueling)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Assume 0.5% of  account 20 - need to add handling for this in MOUSE script.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Spare Parts (Except Manufacturing and Fueling)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Assume 5% of  account 20 - need to confirm handling for this in MOUSE script.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Utilities except electricity, Supplies, and Consumables</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Assume 1% of  account 20 - need to confirm handling for this in MOUSE script.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Electricity</x:t>
   </x:si>
   <x:si>
@@ -2879,9 +2858,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Annualized Transportation Costs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Assume 5% of the sum of accounts 741 and 742 - need to add handling for this in MOUSE script.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Annualized Helium Replenishment</x:t>
@@ -22965,18 +22941,18 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R7ed5c52c791844ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="R0acfdc5f00cd4ce4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="R5396824f765949d6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="Ra383cd6292514a11"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="Rb72f3fa1204e454b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U106" r:id="R9f97213bb1894a5a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U117" r:id="R02e29dab23c54eeb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U127" r:id="Rd484ac8b64754e91"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U128" r:id="R5eeedc6b469f4d83"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U132" r:id="R3d9388127e1a44dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U133" r:id="R46ced60c15d04f34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U166" r:id="Rc38972d7745c49db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R4e34538ee20e4dd9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="R25d545ab52c34ad3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="R7f23699584504f6f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U33" r:id="R0650ebc791c44e3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U49" r:id="R2e755327054d4164"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U106" r:id="Rb29bb72a37654430"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U117" r:id="Rafe5112e87df428f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U127" r:id="R60f0aad1c80745a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U128" r:id="Rdb6659e1fc664996"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U132" r:id="R6f243f268fe64141"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U133" r:id="R1d0ac5e68d6e45ce"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U166" r:id="R2bbc1dc3280e4713"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -25821,7 +25797,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f45ce389a984881"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c307435bf6b4c66"/>
 </x:worksheet>
 </file>
 
@@ -25829,11 +25805,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="47.779998779296875" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="11.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="17.780000686645508" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="33.33000183105469" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="47.779998779296875" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="34" customFormat="1">
@@ -26119,6 +26095,123 @@
       <x:c r="C25" s="230"/>
       <x:c r="D25" s="230"/>
       <x:c r="E25" s="230" t="str">
+        <x:v>Annualized other supplies and utilities.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>MFG Account 223 to Reactor OCC per Testing Line Ratio</x:v>
+      </x:c>
+      <x:c r="B26" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26" t="str">
+        <x:v>REVIEW NEEDED: provisional testing-building assumption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>MFG Account 30 to Account 20 Ratio</x:v>
+      </x:c>
+      <x:c r="B27" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27" t="str">
+        <x:v>Account 30 is 50% of direct cost.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>MFG Account 716 to Accounts 711-715 Ratio</x:v>
+      </x:c>
+      <x:c r="B28" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28" t="str">
+        <x:v>Continuing education and retraining.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>MFG Account 717 to Accounts 711-715 Ratio</x:v>
+      </x:c>
+      <x:c r="B29" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29" t="str">
+        <x:v>Management staff.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>MFG Account 741 to Account 20 Ratio</x:v>
+      </x:c>
+      <x:c r="B30" t="n">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30" t="str">
+        <x:v>Operating chemicals and lubricants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>MFG Account 742 to Account 20 Ratio</x:v>
+      </x:c>
+      <x:c r="B31" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31" t="str">
+        <x:v>Spare parts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>MFG Account 743 to Account 20 Ratio</x:v>
+      </x:c>
+      <x:c r="B32" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32" t="str">
+        <x:v>Utilities excluding electricity, supplies, and consumables.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>MFG Account 747.1 to Accounts 741-743 Ratio</x:v>
+      </x:c>
+      <x:c r="B33" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33" t="str">
+        <x:v>Annualized transportation costs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>MFG Account 747.4 to Account 20 Ratio</x:v>
+      </x:c>
+      <x:c r="B34" t="n">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34" t="str">
         <x:v>Annualized other supplies and utilities.</x:v>
       </x:c>
     </x:row>
@@ -26745,13 +26838,13 @@
       <x:c r="W7" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X7" s="107">
+      <x:c r="X7" s="107" t="n">
         <x:f t="shared" si="4"/>
-        <x:v>11723514.75</x:v>
-      </x:c>
-      <x:c r="Y7" s="107">
+        <x:v>46894059</x:v>
+      </x:c>
+      <x:c r="Y7" s="107" t="n">
         <x:f t="shared" si="5"/>
-        <x:v>19539191.25</x:v>
+        <x:v>78156765</x:v>
       </x:c>
       <x:c r="Z7" s="99" t="s">
         <x:v>44</x:v>
@@ -27885,9 +27978,7 @@
       <x:c r="J23" s="142"/>
       <x:c r="K23" s="180"/>
       <x:c r="L23" s="168"/>
-      <x:c r="M23" s="187" t="s">
-        <x:v>598</x:v>
-      </x:c>
+      <x:c r="M23" s="187"/>
       <x:c r="N23" s="168"/>
       <x:c r="O23" s="168"/>
       <x:c r="P23" s="182"/>
@@ -27951,7 +28042,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C24" s="176" t="s">
-        <x:v>599</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="D24" s="177" t="str">
         <x:f>REPT("   ", B24*2) &amp; C24</x:f>
@@ -27972,7 +28063,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M24" s="181" t="s">
-        <x:v>600</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="N24" s="168">
         <x:v>1</x:v>
@@ -28047,7 +28138,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C25" s="176" t="s">
-        <x:v>601</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="D25" s="177" t="str">
         <x:f t="shared" ref="D25" si="19">REPT("   ", B25*2) &amp; C25</x:f>
@@ -28069,7 +28160,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M25" s="181" t="s">
-        <x:v>602</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="N25" s="168">
         <x:v>1</x:v>
@@ -28183,7 +28274,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C27" s="101" t="s">
-        <x:v>603</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D27" s="96" t="str">
         <x:f>REPT("   ", B27*2) &amp; C27</x:f>
@@ -28193,7 +28284,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F27" s="96" t="s">
-        <x:v>604</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="G27" s="97">
         <x:v>1</x:v>
@@ -28281,7 +28372,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C28" s="194" t="s">
-        <x:v>605</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="D28" s="96" t="str">
         <x:f t="shared" ref="D28:D69" si="25">REPT("   ", B28*2) &amp; C28</x:f>
@@ -28333,7 +28424,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C29" s="176" t="s">
-        <x:v>606</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="D29" s="177" t="str">
         <x:f>REPT("   ", B29*2) &amp; C29</x:f>
@@ -28355,7 +28446,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M29" s="181" t="s">
-        <x:v>607</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="N29" s="168">
         <x:v>1</x:v>
@@ -28369,9 +28460,11 @@
       <x:c r="Q29" s="104">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="R29" s="143"/>
+      <x:c r="R29" s="143" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
       <x:c r="S29" s="196" t="s">
-        <x:v>608</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="T29" s="196"/>
       <x:c r="U29" s="197"/>
@@ -28404,7 +28497,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="176" t="s">
-        <x:v>609</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="D30" s="177" t="str">
         <x:f>REPT("   ", B30*2) &amp; C30</x:f>
@@ -28414,7 +28507,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F30" s="177" t="s">
-        <x:v>610</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="G30" s="179">
         <x:v>1</x:v>
@@ -28497,7 +28590,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C31" s="176" t="s">
-        <x:v>611</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="D31" s="177" t="str">
         <x:f t="shared" ref="D31" si="27">REPT("   ", B31*2) &amp; C31</x:f>
@@ -28519,7 +28612,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M31" s="181" t="s">
-        <x:v>612</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="N31" s="168">
         <x:v>1</x:v>
@@ -28596,7 +28689,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C32" s="176" t="s">
-        <x:v>613</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D32" s="177" t="str">
         <x:f>REPT("   ", B32*2) &amp; C32</x:f>
@@ -28618,7 +28711,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M32" s="181" t="s">
-        <x:v>614</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="N32" s="168">
         <x:v>300</x:v>
@@ -28636,7 +28729,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S32" s="170" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="T32" s="105"/>
       <x:c r="U32" s="157"/>
@@ -28688,7 +28781,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C33" s="194" t="s">
-        <x:v>616</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="D33" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -28733,7 +28826,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C34" s="194" t="s">
-        <x:v>617</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="D34" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -28743,7 +28836,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F34" s="96" t="s">
-        <x:v>618</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="G34" s="97">
         <x:v>1</x:v>
@@ -28766,10 +28859,10 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S34" s="113" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="T34" s="113" t="s">
         <x:v>619</x:v>
-      </x:c>
-      <x:c r="T34" s="113" t="s">
-        <x:v>620</x:v>
       </x:c>
       <x:c r="U34" s="106"/>
       <x:c r="V34" s="106"/>
@@ -28820,7 +28913,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C35" s="194" t="s">
-        <x:v>621</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="D35" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -28830,7 +28923,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F35" s="96" t="s">
-        <x:v>622</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="G35" s="97">
         <x:v>1</x:v>
@@ -28853,7 +28946,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S35" s="113" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T35" s="113"/>
       <x:c r="U35" s="106"/>
@@ -28905,7 +28998,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C36" s="194" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="D36" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -28926,7 +29019,7 @@
       <x:c r="Q36" s="104"/>
       <x:c r="R36" s="106"/>
       <x:c r="S36" s="200" t="s">
-        <x:v>625</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="T36" s="113"/>
       <x:c r="U36" s="201"/>
@@ -28951,7 +29044,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C37" s="194" t="s">
-        <x:v>626</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D37" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -28973,7 +29066,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M37" s="204" t="s">
-        <x:v>627</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="N37" s="106">
         <x:v>1068</x:v>
@@ -28985,9 +29078,11 @@
       <x:c r="Q37" s="104">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="R37" s="106"/>
+      <x:c r="R37" s="106" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
       <x:c r="S37" s="155" t="s">
-        <x:v>628</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="T37" s="113"/>
       <x:c r="U37" s="201"/>
@@ -29012,7 +29107,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C38" s="194" t="s">
-        <x:v>629</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="D38" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29022,7 +29117,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F38" s="96" t="s">
-        <x:v>630</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="G38" s="97">
         <x:v>1</x:v>
@@ -29041,9 +29136,11 @@
       <x:c r="Q38" s="104">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="R38" s="106"/>
+      <x:c r="R38" s="106" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
       <x:c r="S38" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T38" s="113"/>
       <x:c r="U38" s="201"/>
@@ -29068,7 +29165,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C39" s="194" t="s">
-        <x:v>632</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="D39" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29078,7 +29175,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F39" s="96" t="s">
-        <x:v>633</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="G39" s="97">
         <x:v>1</x:v>
@@ -29097,9 +29194,11 @@
       <x:c r="Q39" s="104">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="R39" s="106"/>
+      <x:c r="R39" s="106" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
       <x:c r="S39" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T39" s="113"/>
       <x:c r="U39" s="201"/>
@@ -29124,7 +29223,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C40" s="194" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="D40" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29134,7 +29233,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F40" s="96" t="s">
-        <x:v>635</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="G40" s="97">
         <x:v>1</x:v>
@@ -29153,9 +29252,11 @@
       <x:c r="Q40" s="104">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="R40" s="106"/>
+      <x:c r="R40" s="106" t="str">
+        <x:v>Equipment</x:v>
+      </x:c>
       <x:c r="S40" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T40" s="113"/>
       <x:c r="U40" s="201"/>
@@ -29199,9 +29300,7 @@
       <x:c r="G41" s="97"/>
       <x:c r="H41" s="96"/>
       <x:c r="I41" s="96"/>
-      <x:c r="J41" s="207" t="s">
-        <x:v>636</x:v>
-      </x:c>
+      <x:c r="J41" s="207"/>
       <x:c r="K41" s="108"/>
       <x:c r="L41" s="90"/>
       <x:c r="M41" s="90"/>
@@ -29309,7 +29408,9 @@
       <x:c r="Q43" s="104">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="R43" s="106"/>
+      <x:c r="R43" s="106" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
       <x:c r="S43" s="113"/>
       <x:c r="T43" s="106"/>
       <x:c r="U43" s="106"/>
@@ -29541,7 +29642,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="112" t="s">
-        <x:v>637</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="D48" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29562,7 +29663,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M48" s="113" t="s">
-        <x:v>638</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="N48" s="106"/>
       <x:c r="O48" s="106"/>
@@ -29628,7 +29729,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C49" s="112" t="s">
-        <x:v>639</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="D49" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29649,7 +29750,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M49" s="59" t="s">
-        <x:v>640</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="N49" s="106"/>
       <x:c r="O49" s="106"/>
@@ -29663,10 +29764,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="S49" s="59" t="s">
-        <x:v>641</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="T49" s="59" t="s">
-        <x:v>642</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="U49" s="106"/>
       <x:c r="V49" s="106"/>
@@ -29738,7 +29839,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M50" s="59" t="s">
-        <x:v>643</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="N50" s="106"/>
       <x:c r="O50" s="106"/>
@@ -29804,7 +29905,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C51" s="112" t="s">
-        <x:v>644</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="D51" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29825,7 +29926,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M51" s="59" t="s">
-        <x:v>645</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="N51" s="106"/>
       <x:c r="O51" s="106"/>
@@ -29891,7 +29992,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C52" s="112" t="s">
-        <x:v>646</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="D52" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29912,7 +30013,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M52" s="209" t="s">
-        <x:v>647</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="N52" s="106"/>
       <x:c r="O52" s="106"/>
@@ -29974,7 +30075,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C53" s="112" t="s">
-        <x:v>648</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="D53" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -29985,9 +30086,7 @@
       <x:c r="G53" s="97"/>
       <x:c r="H53" s="96"/>
       <x:c r="I53" s="96"/>
-      <x:c r="J53" s="207" t="s">
-        <x:v>649</x:v>
-      </x:c>
+      <x:c r="J53" s="207"/>
       <x:c r="K53" s="61"/>
       <x:c r="L53" s="49"/>
       <x:c r="M53" s="59"/>
@@ -30005,13 +30104,11 @@
       <x:c r="W53" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X53" s="107" t="e">
+      <x:c r="X53" s="107">
         <x:f t="shared" si="36"/>
-        <x:v>#VALUE!</x:v>
-      </x:c>
-      <x:c r="Y53" s="107" t="e">
+      </x:c>
+      <x:c r="Y53" s="107">
         <x:f t="shared" si="37"/>
-        <x:v>#VALUE!</x:v>
       </x:c>
       <x:c r="Z53" s="99" t="s">
         <x:v>44</x:v>
@@ -30049,7 +30146,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C54" s="112" t="s">
-        <x:v>650</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="D54" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30060,9 +30157,7 @@
       <x:c r="G54" s="97"/>
       <x:c r="H54" s="96"/>
       <x:c r="I54" s="96"/>
-      <x:c r="J54" s="207" t="s">
-        <x:v>651</x:v>
-      </x:c>
+      <x:c r="J54" s="207"/>
       <x:c r="K54" s="210"/>
       <x:c r="L54" s="211"/>
       <x:c r="M54" s="212"/>
@@ -30080,13 +30175,11 @@
       <x:c r="W54" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X54" s="107" t="e">
+      <x:c r="X54" s="107">
         <x:f t="shared" si="36"/>
-        <x:v>#VALUE!</x:v>
-      </x:c>
-      <x:c r="Y54" s="107" t="e">
+      </x:c>
+      <x:c r="Y54" s="107">
         <x:f t="shared" si="37"/>
-        <x:v>#VALUE!</x:v>
       </x:c>
       <x:c r="Z54" s="99" t="s">
         <x:v>44</x:v>
@@ -30124,7 +30217,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C55" s="112" t="s">
-        <x:v>652</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="D55" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30213,7 +30306,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C56" s="112" t="s">
-        <x:v>653</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="D56" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30302,7 +30395,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C57" s="112" t="s">
-        <x:v>654</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="D57" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30347,7 +30440,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C58" s="112" t="s">
-        <x:v>655</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="D58" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30358,9 +30451,7 @@
       <x:c r="G58" s="97"/>
       <x:c r="H58" s="96"/>
       <x:c r="I58" s="96"/>
-      <x:c r="J58" s="207" t="s">
-        <x:v>656</x:v>
-      </x:c>
+      <x:c r="J58" s="207"/>
       <x:c r="K58" s="102"/>
       <x:c r="L58" s="106"/>
       <x:c r="M58" s="113"/>
@@ -30376,13 +30467,11 @@
       <x:c r="W58" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X58" s="107" t="e">
+      <x:c r="X58" s="107">
         <x:f t="shared" si="36"/>
-        <x:v>#VALUE!</x:v>
-      </x:c>
-      <x:c r="Y58" s="107" t="e">
+      </x:c>
+      <x:c r="Y58" s="107">
         <x:f t="shared" ref="Y58:Y64" si="40">1.5*J58</x:f>
-        <x:v>#VALUE!</x:v>
       </x:c>
       <x:c r="Z58" s="99" t="s">
         <x:v>44</x:v>
@@ -30420,7 +30509,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C59" s="112" t="s">
-        <x:v>657</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="D59" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30431,9 +30520,7 @@
       <x:c r="G59" s="97"/>
       <x:c r="H59" s="96"/>
       <x:c r="I59" s="96"/>
-      <x:c r="J59" s="207" t="s">
-        <x:v>658</x:v>
-      </x:c>
+      <x:c r="J59" s="207"/>
       <x:c r="K59" s="102"/>
       <x:c r="L59" s="106"/>
       <x:c r="M59" s="113"/>
@@ -30449,13 +30536,11 @@
       <x:c r="W59" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X59" s="107" t="e">
+      <x:c r="X59" s="107">
         <x:f t="shared" si="36"/>
-        <x:v>#VALUE!</x:v>
-      </x:c>
-      <x:c r="Y59" s="107" t="e">
+      </x:c>
+      <x:c r="Y59" s="107">
         <x:f t="shared" si="40"/>
-        <x:v>#VALUE!</x:v>
       </x:c>
       <x:c r="Z59" s="99" t="s">
         <x:v>44</x:v>
@@ -30493,7 +30578,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C60" s="112" t="s">
-        <x:v>659</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="D60" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30504,9 +30589,7 @@
       <x:c r="G60" s="97"/>
       <x:c r="H60" s="96"/>
       <x:c r="I60" s="96"/>
-      <x:c r="J60" s="207" t="s">
-        <x:v>660</x:v>
-      </x:c>
+      <x:c r="J60" s="207"/>
       <x:c r="K60" s="102"/>
       <x:c r="L60" s="106"/>
       <x:c r="M60" s="113"/>
@@ -30522,13 +30605,11 @@
       <x:c r="W60" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X60" s="107" t="e">
+      <x:c r="X60" s="107">
         <x:f t="shared" si="36"/>
-        <x:v>#VALUE!</x:v>
-      </x:c>
-      <x:c r="Y60" s="107" t="e">
+      </x:c>
+      <x:c r="Y60" s="107">
         <x:f t="shared" si="40"/>
-        <x:v>#VALUE!</x:v>
       </x:c>
       <x:c r="Z60" s="99" t="s">
         <x:v>44</x:v>
@@ -30566,7 +30647,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C61" s="112" t="s">
-        <x:v>661</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="D61" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30601,7 +30682,9 @@
       <x:c r="Q61" s="104">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="R61" s="106"/>
+      <x:c r="R61" s="106" t="str">
+        <x:v>General</x:v>
+      </x:c>
       <x:c r="S61" s="113"/>
       <x:c r="T61" s="114"/>
       <x:c r="U61" s="208"/>
@@ -30653,7 +30736,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C62" s="112" t="s">
-        <x:v>662</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="D62" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30742,7 +30825,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C63" s="112" t="s">
-        <x:v>663</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="D63" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30831,7 +30914,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C64" s="112" t="s">
-        <x:v>664</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="D64" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30902,7 +30985,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C65" s="112" t="s">
-        <x:v>665</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="D65" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30913,9 +30996,7 @@
       <x:c r="G65" s="97"/>
       <x:c r="H65" s="96"/>
       <x:c r="I65" s="96"/>
-      <x:c r="J65" s="207" t="s">
-        <x:v>666</x:v>
-      </x:c>
+      <x:c r="J65" s="207"/>
       <x:c r="K65" s="102"/>
       <x:c r="L65" s="106"/>
       <x:c r="M65" s="113"/>
@@ -30929,13 +31010,11 @@
       <x:c r="U65" s="208"/>
       <x:c r="V65" s="106"/>
       <x:c r="W65" s="99"/>
-      <x:c r="X65" s="107" t="n">
+      <x:c r="X65" s="107">
         <x:f t="shared" ref="X65" si="43">0.8*$I65</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Y65" s="107" t="e">
+      </x:c>
+      <x:c r="Y65" s="107">
         <x:f t="shared" ref="Y65" si="44">2*J65</x:f>
-        <x:v>#VALUE!</x:v>
       </x:c>
       <x:c r="Z65" s="99" t="s">
         <x:v>44</x:v>
@@ -30973,7 +31052,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C66" s="112" t="s">
-        <x:v>667</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="D66" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -30998,7 +31077,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M66" s="209" t="s">
-        <x:v>668</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="N66" s="106"/>
       <x:c r="O66" s="106" t="s">
@@ -31068,7 +31147,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C67" s="112" t="s">
-        <x:v>669</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="D67" s="96" t="str">
         <x:f t="shared" si="25"/>
@@ -31079,9 +31158,7 @@
       <x:c r="G67" s="97"/>
       <x:c r="H67" s="96"/>
       <x:c r="I67" s="96"/>
-      <x:c r="J67" s="207" t="s">
-        <x:v>656</x:v>
-      </x:c>
+      <x:c r="J67" s="207"/>
       <x:c r="K67" s="102"/>
       <x:c r="L67" s="106"/>
       <x:c r="M67" s="113"/>
@@ -31097,12 +31174,8 @@
       <x:c r="W67" s="99" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="X67" s="107">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Y67" s="107">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="X67" s="107"/>
+      <x:c r="Y67" s="107"/>
       <x:c r="Z67" s="99" t="s">
         <x:v>44</x:v>
       </x:c>
@@ -31504,12 +31577,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R146889ef723144a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="R4ee23c77680d4c4d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U66" r:id="R8f7d05aedf164762"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R8dc222345a254d6f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="R66ade67c7e39413b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U66" r:id="R717fafed3b4944ec"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc4565902e5e49fc"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4dad1a1980494c"/>
 </x:worksheet>
 </file>
 
@@ -31741,7 +31814,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M3" s="103" t="s">
-        <x:v>670</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="N3" s="143"/>
       <x:c r="O3" s="103" t="s">
@@ -31837,7 +31910,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M4" s="103" t="s">
-        <x:v>671</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="N4" s="143"/>
       <x:c r="O4" s="103" t="s">
@@ -32340,7 +32413,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M11" s="103" t="s">
-        <x:v>672</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="N11" s="143"/>
       <x:c r="O11" s="103" t="s">
@@ -32443,7 +32516,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M12" s="103" t="s">
-        <x:v>672</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="N12" s="143"/>
       <x:c r="O12" s="103" t="s">
@@ -32533,7 +32606,7 @@
         <x:v>578</x:v>
       </x:c>
       <x:c r="M13" s="149" t="s">
-        <x:v>673</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="N13" s="150">
         <x:v>1</x:v>
@@ -32672,7 +32745,7 @@
         <x:v>583</x:v>
       </x:c>
       <x:c r="M15" s="103" t="s">
-        <x:v>674</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="N15" s="143"/>
       <x:c r="O15" s="103"/>
@@ -32736,7 +32809,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C16" s="101" t="s">
-        <x:v>675</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="D16" s="96" t="str">
         <x:f t="shared" si="1"/>
@@ -32762,7 +32835,7 @@
         <x:v>583</x:v>
       </x:c>
       <x:c r="M16" s="103" t="s">
-        <x:v>676</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="N16" s="143"/>
       <x:c r="O16" s="103"/>
@@ -32852,7 +32925,7 @@
         <x:v>583</x:v>
       </x:c>
       <x:c r="M17" s="103" t="s">
-        <x:v>677</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="N17" s="143"/>
       <x:c r="O17" s="103"/>
@@ -32961,7 +33034,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="101" t="s">
-        <x:v>678</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="D19" s="96" t="str">
         <x:f t="shared" si="1"/>
@@ -33006,7 +33079,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="176" t="s">
-        <x:v>679</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="D20" s="177" t="str">
         <x:f t="shared" si="1"/>
@@ -33032,7 +33105,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M20" s="181" t="s">
-        <x:v>680</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="N20" s="168" t="n">
         <x:f>338988/(3.2808^2)</x:f>
@@ -33051,7 +33124,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S20" s="170" t="s">
-        <x:v>681</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="T20" s="196"/>
       <x:c r="U20" s="197"/>
@@ -33103,7 +33176,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C21" s="101" t="s">
-        <x:v>682</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="D21" s="96"/>
       <x:c r="E21" s="96"/>
@@ -33145,7 +33218,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C22" s="176" t="s">
-        <x:v>683</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="D22" s="177" t="str">
         <x:f t="shared" ref="D22" si="13">REPT("   ", B22*2) &amp; C22</x:f>
@@ -33171,7 +33244,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M22" s="181" t="s">
-        <x:v>684</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="N22" s="168">
         <x:v>1</x:v>
@@ -33189,7 +33262,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S22" s="170" t="s">
-        <x:v>685</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="T22" s="196"/>
       <x:c r="U22" s="197"/>
@@ -33292,7 +33365,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C24" s="101" t="s">
-        <x:v>686</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="D24" s="96" t="str">
         <x:f t="shared" ref="D24:D31" si="18">REPT("   ", B24*2) &amp; C24</x:f>
@@ -33318,7 +33391,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M24" s="101" t="s">
-        <x:v>687</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="N24" s="168">
         <x:v>1</x:v>
@@ -33387,7 +33460,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C25" s="101" t="s">
-        <x:v>688</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="D25" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33413,7 +33486,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M25" s="101" t="s">
-        <x:v>689</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="N25" s="168">
         <x:v>1</x:v>
@@ -33490,7 +33563,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C26" s="101" t="s">
-        <x:v>690</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D26" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33535,7 +33608,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C27" s="101" t="s">
-        <x:v>691</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="D27" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33561,7 +33634,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M27" s="181" t="s">
-        <x:v>692</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="N27" s="168">
         <x:v>1</x:v>
@@ -33579,7 +33652,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S27" s="170" t="s">
-        <x:v>685</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="T27" s="105"/>
       <x:c r="U27" s="157"/>
@@ -33631,7 +33704,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C28" s="101" t="s">
-        <x:v>693</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="D28" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33653,7 +33726,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M28" s="181" t="s">
-        <x:v>694</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="N28" s="143">
         <x:v>1</x:v>
@@ -33671,11 +33744,11 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S28" s="105" t="s">
-        <x:v>695</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="T28" s="105"/>
       <x:c r="U28" s="166" t="s">
-        <x:v>696</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="V28" s="106"/>
       <x:c r="W28" s="171" t="s">
@@ -33725,7 +33798,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C29" s="101" t="s">
-        <x:v>697</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="D29" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33747,7 +33820,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M29" s="181" t="s">
-        <x:v>698</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="N29" s="143">
         <x:v>1</x:v>
@@ -33765,7 +33838,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S29" s="170" t="s">
-        <x:v>685</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="T29" s="105"/>
       <x:c r="U29" s="157"/>
@@ -33817,7 +33890,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="101" t="s">
-        <x:v>699</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D30" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33862,7 +33935,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="101" t="s">
-        <x:v>700</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="D31" s="96" t="str">
         <x:f t="shared" si="18"/>
@@ -33891,7 +33964,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S31" s="170" t="s">
-        <x:v>701</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="T31" s="105"/>
       <x:c r="U31" s="157"/>
@@ -33987,7 +34060,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C33" s="176" t="s">
-        <x:v>702</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D33" s="177" t="str">
         <x:f>REPT("   ", B33*2) &amp; C33</x:f>
@@ -34007,7 +34080,7 @@
       </x:c>
       <x:c r="L33" s="168"/>
       <x:c r="M33" s="181" t="s">
-        <x:v>703</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="N33" s="168">
         <x:v>300</x:v>
@@ -34025,7 +34098,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S33" s="170" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="T33" s="105"/>
       <x:c r="U33" s="157"/>
@@ -34084,7 +34157,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C34" s="176" t="s">
-        <x:v>704</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="D34" s="177" t="str">
         <x:f>REPT("   ", B34*2) &amp; C34</x:f>
@@ -34104,7 +34177,7 @@
       </x:c>
       <x:c r="L34" s="168"/>
       <x:c r="M34" s="181" t="s">
-        <x:v>703</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="N34" s="168">
         <x:v>300</x:v>
@@ -34122,7 +34195,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S34" s="170" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="T34" s="105"/>
       <x:c r="U34" s="157"/>
@@ -34181,7 +34254,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C35" s="176" t="s">
-        <x:v>705</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="D35" s="177" t="str">
         <x:f>REPT("   ", B35*2) &amp; C35</x:f>
@@ -34202,7 +34275,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M35" s="181" t="s">
-        <x:v>706</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="N35" s="168">
         <x:v>1</x:v>
@@ -34277,7 +34350,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C36" s="176" t="s">
-        <x:v>601</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="D36" s="177" t="str">
         <x:f t="shared" ref="D36" si="34">REPT("   ", B36*2) &amp; C36</x:f>
@@ -34299,7 +34372,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M36" s="181" t="s">
-        <x:v>707</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="N36" s="168">
         <x:v>1</x:v>
@@ -34413,7 +34486,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C38" s="101" t="s">
-        <x:v>708</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="D38" s="96" t="str">
         <x:f>REPT("   ", B38*2) &amp; C38</x:f>
@@ -34423,7 +34496,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F38" s="96" t="s">
-        <x:v>709</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="G38" s="97">
         <x:v>1</x:v>
@@ -34446,7 +34519,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S38" s="146" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T38" s="105"/>
       <x:c r="U38" s="157"/>
@@ -34497,7 +34570,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C39" s="176" t="s">
-        <x:v>710</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="D39" s="177" t="str">
         <x:f t="shared" ref="D39" si="35">REPT("   ", B39*2) &amp; C39</x:f>
@@ -34521,7 +34594,7 @@
       </x:c>
       <x:c r="L39" s="168"/>
       <x:c r="M39" s="181" t="s">
-        <x:v>711</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="N39" s="224" t="n">
         <x:f>200/3600</x:f>
@@ -34540,10 +34613,10 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S39" s="170" t="s">
-        <x:v>712</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="T39" s="196" t="s">
-        <x:v>713</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="U39" s="197" t="s">
         <x:v>306</x:v>
@@ -34595,7 +34668,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C40" s="101" t="s">
-        <x:v>714</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="D40" s="96" t="str">
         <x:f>REPT("   ", B40*2) &amp; C40</x:f>
@@ -34605,7 +34678,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F40" s="96" t="s">
-        <x:v>715</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="G40" s="97">
         <x:v>1</x:v>
@@ -34628,12 +34701,12 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S40" s="105" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T40" s="105"/>
       <x:c r="U40" s="157"/>
       <x:c r="V40" s="106" t="s">
-        <x:v>716</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="W40" s="99" t="s">
         <x:v>43</x:v>
@@ -34681,7 +34754,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C41" s="101" t="s">
-        <x:v>603</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D41" s="96" t="str">
         <x:f>REPT("   ", B41*2) &amp; C41</x:f>
@@ -34691,7 +34764,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F41" s="96" t="s">
-        <x:v>709</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="G41" s="97">
         <x:v>1</x:v>
@@ -34715,13 +34788,13 @@
         <x:v>Lab and Mat and Equip</x:v>
       </x:c>
       <x:c r="S41" s="105" t="s">
-        <x:v>717</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="T41" s="105" t="s">
-        <x:v>718</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="U41" s="166" t="s">
-        <x:v>719</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="V41" s="106"/>
       <x:c r="W41" s="171" t="s">
@@ -34770,7 +34843,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C42" s="101" t="s">
-        <x:v>720</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="D42" s="96" t="str">
         <x:f>REPT("   ", B42*2) &amp; C42</x:f>
@@ -34793,7 +34866,7 @@
       </x:c>
       <x:c r="L42" s="103"/>
       <x:c r="M42" s="96" t="s">
-        <x:v>721</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="N42" s="143"/>
       <x:c r="O42" s="103"/>
@@ -34805,7 +34878,7 @@
         <x:v>Lab and Mat and Equip</x:v>
       </x:c>
       <x:c r="S42" s="105" t="s">
-        <x:v>722</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="T42" s="105"/>
       <x:c r="U42" s="157"/>
@@ -34856,7 +34929,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C43" s="101" t="s">
-        <x:v>723</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="D43" s="96" t="str">
         <x:f>REPT("   ", B43*2) &amp; C43</x:f>
@@ -34879,7 +34952,7 @@
       <x:c r="K43" s="142"/>
       <x:c r="L43" s="103"/>
       <x:c r="M43" s="96" t="s">
-        <x:v>724</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="N43" s="143"/>
       <x:c r="O43" s="103"/>
@@ -34891,7 +34964,7 @@
         <x:v>Lab and Mat and Equip</x:v>
       </x:c>
       <x:c r="S43" s="105" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T43" s="105"/>
       <x:c r="U43" s="157"/>
@@ -34950,7 +35023,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C44" s="194" t="s">
-        <x:v>605</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="D44" s="96" t="str">
         <x:f t="shared" ref="D44:D99" si="44">REPT("   ", B44*2) &amp; C44</x:f>
@@ -35002,7 +35075,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C45" s="176" t="s">
-        <x:v>606</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="D45" s="177" t="str">
         <x:f>REPT("   ", B45*2) &amp; C45</x:f>
@@ -35024,7 +35097,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M45" s="181" t="s">
-        <x:v>725</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="N45" s="168">
         <x:v>1</x:v>
@@ -35042,7 +35115,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S45" s="196" t="s">
-        <x:v>608</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="T45" s="196"/>
       <x:c r="U45" s="197"/>
@@ -35101,7 +35174,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C46" s="176" t="s">
-        <x:v>726</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="D46" s="177" t="str">
         <x:f>REPT("   ", B46*2) &amp; C46</x:f>
@@ -35111,7 +35184,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F46" s="177" t="s">
-        <x:v>727</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="G46" s="179">
         <x:v>1</x:v>
@@ -35134,7 +35207,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S46" s="170" t="s">
-        <x:v>685</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="T46" s="105"/>
       <x:c r="U46" s="157"/>
@@ -35193,7 +35266,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C47" s="176" t="s">
-        <x:v>609</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="D47" s="177" t="str">
         <x:f t="shared" ref="D47:D48" si="49">REPT("   ", B47*2) &amp; C47</x:f>
@@ -35203,7 +35276,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F47" s="177" t="s">
-        <x:v>728</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="G47" s="179">
         <x:v>1</x:v>
@@ -35279,7 +35352,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="176" t="s">
-        <x:v>611</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="D48" s="177" t="str">
         <x:f t="shared" si="49"/>
@@ -35301,7 +35374,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="M48" s="181" t="s">
-        <x:v>729</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="N48" s="168">
         <x:v>1</x:v>
@@ -35378,7 +35451,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C49" s="176" t="s">
-        <x:v>613</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D49" s="177" t="str">
         <x:f>REPT("   ", B49*2) &amp; C49</x:f>
@@ -35400,7 +35473,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M49" s="181" t="s">
-        <x:v>671</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="N49" s="168">
         <x:v>300</x:v>
@@ -35418,7 +35491,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="S49" s="170" t="s">
-        <x:v>615</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="T49" s="105"/>
       <x:c r="U49" s="157"/>
@@ -35470,7 +35543,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C50" s="194" t="s">
-        <x:v>616</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="D50" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35515,7 +35588,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C51" s="194" t="s">
-        <x:v>617</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="D51" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35525,7 +35598,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F51" s="96" t="s">
-        <x:v>730</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="G51" s="97">
         <x:v>1</x:v>
@@ -35548,10 +35621,10 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S51" s="113" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="T51" s="113" t="s">
         <x:v>619</x:v>
-      </x:c>
-      <x:c r="T51" s="113" t="s">
-        <x:v>620</x:v>
       </x:c>
       <x:c r="U51" s="106"/>
       <x:c r="V51" s="106"/>
@@ -35602,7 +35675,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C52" s="194" t="s">
-        <x:v>621</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="D52" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35612,7 +35685,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F52" s="96" t="s">
-        <x:v>731</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="G52" s="97">
         <x:v>1</x:v>
@@ -35635,7 +35708,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S52" s="113" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T52" s="113"/>
       <x:c r="U52" s="106"/>
@@ -35687,7 +35760,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C53" s="194" t="s">
-        <x:v>732</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="D53" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35732,7 +35805,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C54" s="194" t="s">
-        <x:v>733</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="D54" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35742,7 +35815,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F54" s="96" t="s">
-        <x:v>734</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="G54" s="97">
         <x:v>1</x:v>
@@ -35765,7 +35838,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S54" s="113" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T54" s="113"/>
       <x:c r="U54" s="226"/>
@@ -35817,7 +35890,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C55" s="194" t="s">
-        <x:v>735</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="D55" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35827,7 +35900,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F55" s="96" t="s">
-        <x:v>736</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="G55" s="97">
         <x:v>1</x:v>
@@ -35850,7 +35923,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S55" s="113" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T55" s="113"/>
       <x:c r="U55" s="226"/>
@@ -35902,7 +35975,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C56" s="194" t="s">
-        <x:v>737</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="D56" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35912,7 +35985,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F56" s="96" t="s">
-        <x:v>738</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="G56" s="97">
         <x:v>1</x:v>
@@ -35935,7 +36008,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S56" s="113" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T56" s="113"/>
       <x:c r="U56" s="226"/>
@@ -35987,7 +36060,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C57" s="194" t="s">
-        <x:v>739</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="D57" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -35997,7 +36070,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F57" s="96" t="s">
-        <x:v>740</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="G57" s="97">
         <x:v>1</x:v>
@@ -36020,7 +36093,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S57" s="113" t="s">
-        <x:v>623</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="T57" s="113"/>
       <x:c r="U57" s="226"/>
@@ -36072,7 +36145,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C58" s="194" t="s">
-        <x:v>741</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="D58" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36117,7 +36190,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C59" s="194" t="s">
-        <x:v>742</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="D59" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36127,7 +36200,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F59" s="96" t="s">
-        <x:v>743</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="G59" s="97">
         <x:v>1</x:v>
@@ -36150,7 +36223,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S59" s="113" t="s">
-        <x:v>701</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="T59" s="113"/>
       <x:c r="U59" s="226"/>
@@ -36202,7 +36275,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C60" s="194" t="s">
-        <x:v>744</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="D60" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36235,7 +36308,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S60" s="113" t="s">
-        <x:v>701</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="T60" s="113"/>
       <x:c r="U60" s="226"/>
@@ -36287,7 +36360,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C61" s="194" t="s">
-        <x:v>624</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="D61" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36308,7 +36381,7 @@
       <x:c r="Q61" s="104"/>
       <x:c r="R61" s="106"/>
       <x:c r="S61" s="200" t="s">
-        <x:v>625</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="T61" s="113"/>
       <x:c r="U61" s="201"/>
@@ -36333,7 +36406,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C62" s="194" t="s">
-        <x:v>626</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="D62" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36355,7 +36428,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="M62" s="204" t="s">
-        <x:v>672</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="N62" s="106">
         <x:v>1068</x:v>
@@ -36371,7 +36444,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S62" s="155" t="s">
-        <x:v>628</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="T62" s="113"/>
       <x:c r="U62" s="201"/>
@@ -36422,7 +36495,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C63" s="194" t="s">
-        <x:v>629</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="D63" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36432,7 +36505,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F63" s="96" t="s">
-        <x:v>745</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="G63" s="97">
         <x:v>1</x:v>
@@ -36455,7 +36528,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S63" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T63" s="113"/>
       <x:c r="U63" s="201"/>
@@ -36506,7 +36579,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C64" s="194" t="s">
-        <x:v>632</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="D64" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36516,7 +36589,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F64" s="96" t="s">
-        <x:v>746</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="G64" s="97">
         <x:v>1</x:v>
@@ -36539,7 +36612,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S64" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T64" s="113"/>
       <x:c r="U64" s="201"/>
@@ -36590,7 +36663,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C65" s="194" t="s">
-        <x:v>634</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="D65" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -36600,7 +36673,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F65" s="96" t="s">
-        <x:v>747</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="G65" s="97">
         <x:v>1</x:v>
@@ -36623,7 +36696,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S65" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T65" s="113"/>
       <x:c r="U65" s="201"/>
@@ -36674,7 +36747,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C66" s="194" t="s">
-        <x:v>748</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="D66" s="96" t="str">
         <x:f>REPT("   ", B66*2) &amp; C66</x:f>
@@ -36684,7 +36757,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F66" s="96" t="s">
-        <x:v>749</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="G66" s="97">
         <x:v>1</x:v>
@@ -36707,7 +36780,7 @@
         <x:v>Equipment</x:v>
       </x:c>
       <x:c r="S66" s="155" t="s">
-        <x:v>631</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="T66" s="113"/>
       <x:c r="U66" s="201"/>
@@ -37129,7 +37202,7 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="F74" s="96" t="s">
-        <x:v>750</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="G74" s="97">
         <x:v>1</x:v>
@@ -37144,7 +37217,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M74" s="113" t="s">
-        <x:v>751</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="N74" s="106"/>
       <x:c r="O74" s="106"/>
@@ -37235,7 +37308,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M75" s="96" t="s">
-        <x:v>721</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="N75" s="106"/>
       <x:c r="O75" s="106"/>
@@ -37311,7 +37384,7 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="F76" s="96" t="s">
-        <x:v>750</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="G76" s="97">
         <x:v>1</x:v>
@@ -37326,7 +37399,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M76" s="59" t="s">
-        <x:v>752</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="N76" s="106"/>
       <x:c r="O76" s="106"/>
@@ -37392,7 +37465,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C77" s="112" t="s">
-        <x:v>644</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="D77" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37402,7 +37475,7 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="F77" s="96" t="s">
-        <x:v>750</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="G77" s="97">
         <x:v>1</x:v>
@@ -37483,7 +37556,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C78" s="112" t="s">
-        <x:v>753</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="D78" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37504,7 +37577,7 @@
         <x:v>386</x:v>
       </x:c>
       <x:c r="M78" s="209" t="s">
-        <x:v>754</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="N78" s="106"/>
       <x:c r="O78" s="106"/>
@@ -37566,7 +37639,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C79" s="112" t="s">
-        <x:v>648</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="D79" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37623,7 +37696,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C80" s="112" t="s">
-        <x:v>650</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="D80" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37680,7 +37753,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C81" s="112" t="s">
-        <x:v>654</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="D81" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37725,7 +37798,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C82" s="112" t="s">
-        <x:v>755</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="D82" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37783,7 +37856,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C83" s="112" t="s">
-        <x:v>756</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="D83" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37838,7 +37911,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C84" s="112" t="s">
-        <x:v>659</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="D84" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37893,7 +37966,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C85" s="112" t="s">
-        <x:v>661</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="D85" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -37918,7 +37991,7 @@
         <x:v>418</x:v>
       </x:c>
       <x:c r="M85" s="96" t="s">
-        <x:v>757</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="N85" s="106"/>
       <x:c r="O85" s="106"/>
@@ -37982,7 +38055,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C86" s="112" t="s">
-        <x:v>665</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="D86" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38041,7 +38114,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C87" s="112" t="s">
-        <x:v>758</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="D87" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38086,7 +38159,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C88" s="112" t="s">
-        <x:v>759</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="D88" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38096,7 +38169,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F88" s="96" t="s">
-        <x:v>760</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="G88" s="97">
         <x:v>1</x:v>
@@ -38119,12 +38192,12 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S88" s="113" t="s">
-        <x:v>761</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="T88" s="114"/>
       <x:c r="U88" s="208"/>
       <x:c r="V88" s="106" t="s">
-        <x:v>762</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="W88" s="99" t="s">
         <x:v>43</x:v>
@@ -38171,7 +38244,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C89" s="112" t="s">
-        <x:v>763</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="D89" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38181,7 +38254,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F89" s="96" t="s">
-        <x:v>764</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="G89" s="97">
         <x:v>1</x:v>
@@ -38276,7 +38349,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C90" s="112" t="s">
-        <x:v>765</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="D90" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38286,7 +38359,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F90" s="96" t="s">
-        <x:v>766</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="G90" s="97">
         <x:v>1</x:v>
@@ -38309,12 +38382,12 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="S90" s="113" t="s">
-        <x:v>761</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="T90" s="114"/>
       <x:c r="U90" s="208"/>
       <x:c r="V90" s="106" t="s">
-        <x:v>762</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="W90" s="99" t="s">
         <x:v>43</x:v>
@@ -38361,7 +38434,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C91" s="112" t="s">
-        <x:v>667</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="D91" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38386,7 +38459,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="M91" s="113" t="s">
-        <x:v>767</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="N91" s="106"/>
       <x:c r="O91" s="106" t="s">
@@ -38456,7 +38529,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C92" s="112" t="s">
-        <x:v>669</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="D92" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38501,7 +38574,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C93" s="112" t="s">
-        <x:v>768</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="D93" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38546,7 +38619,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C94" s="194" t="s">
-        <x:v>769</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="D94" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38556,7 +38629,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F94" s="96" t="s">
-        <x:v>734</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="G94" s="97">
         <x:v>1</x:v>
@@ -38630,7 +38703,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C95" s="194" t="s">
-        <x:v>770</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="D95" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38640,7 +38713,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F95" s="96" t="s">
-        <x:v>736</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="G95" s="97">
         <x:v>1</x:v>
@@ -38714,7 +38787,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C96" s="194" t="s">
-        <x:v>771</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="D96" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38724,7 +38797,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F96" s="96" t="s">
-        <x:v>738</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="G96" s="97">
         <x:v>1</x:v>
@@ -38798,7 +38871,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C97" s="194" t="s">
-        <x:v>772</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="D97" s="96" t="str">
         <x:f t="shared" si="44"/>
@@ -38808,7 +38881,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F97" s="96" t="s">
-        <x:v>740</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="G97" s="97">
         <x:v>1</x:v>
@@ -39252,13 +39325,13 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="Ref510b6a5f354956"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="R96a6c4ae10ed49f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="R15030bf7d56f43fb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="R4992b1fc0893483f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U91" r:id="R95f3a41021bf450c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="R99328aabb8ee4325"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="R6f8e9a9d6fd14c0a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U39" r:id="R9b12061b3491421d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U41" r:id="Rfa08ce41e9104c2d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U91" r:id="R9ad569354bf24571"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdba283c3ed744199"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6948e472f2042a4"/>
 </x:worksheet>
 </file>
</xml_diff>